<commit_message>
Sistem Raporu: Excel listesi şefin güncel dosyası ile otomatik senkronize edildi (TSİ)
</commit_message>
<xml_diff>
--- a/Gorev-Listesi.xlsx
+++ b/Gorev-Listesi.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="135">
   <si>
     <t>CUMA</t>
   </si>
@@ -423,6 +423,12 @@
   </si>
   <si>
     <t>S.ARAS.</t>
+  </si>
+  <si>
+    <t>İLETİŞİM BAŞKANLIĞI</t>
+  </si>
+  <si>
+    <t>S.CÜREBAL.</t>
   </si>
 </sst>
 </file>
@@ -1557,7 +1563,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="223">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2161,12 +2167,6 @@
     <xf numFmtId="49" fontId="8" fillId="9" borderId="16" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="6" borderId="41" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="39" fillId="6" borderId="42" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="37" fillId="9" borderId="8" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2196,6 +2196,33 @@
     </xf>
     <xf numFmtId="0" fontId="37" fillId="9" borderId="13" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="9" borderId="41" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="9" borderId="42" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="9" borderId="43" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="32" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="33" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="34" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="38" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="39" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="9" borderId="40" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="58">
@@ -3153,11 +3180,11 @@
       <c r="AE9" s="129"/>
       <c r="AF9" s="130"/>
       <c r="AG9" s="38"/>
-      <c r="AH9" s="136" t="s">
-        <v>15</v>
-      </c>
-      <c r="AI9" s="137"/>
-      <c r="AJ9" s="138"/>
+      <c r="AH9" s="167" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI9" s="168"/>
+      <c r="AJ9" s="169"/>
       <c r="AK9" s="38"/>
       <c r="AL9" s="136" t="s">
         <v>15</v>
@@ -3206,9 +3233,11 @@
       <c r="AE10" s="174"/>
       <c r="AF10" s="175"/>
       <c r="AG10" s="39"/>
-      <c r="AH10" s="170"/>
-      <c r="AI10" s="171"/>
-      <c r="AJ10" s="172"/>
+      <c r="AH10" s="221" t="s">
+        <v>134</v>
+      </c>
+      <c r="AI10" s="222"/>
+      <c r="AJ10" s="223"/>
       <c r="AK10" s="39"/>
       <c r="AL10" s="170"/>
       <c r="AM10" s="171"/>
@@ -3267,7 +3296,7 @@
       </c>
       <c r="AQ11" s="22">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR11" s="27"/>
     </row>
@@ -4046,10 +4075,10 @@
         <v>34</v>
       </c>
       <c r="AG24" s="38"/>
-      <c r="AH24" s="101" t="s">
-        <v>9</v>
-      </c>
-      <c r="AI24" s="102"/>
+      <c r="AH24" s="103" t="s">
+        <v>11</v>
+      </c>
+      <c r="AI24" s="104"/>
       <c r="AJ24" s="56" t="s">
         <v>34</v>
       </c>
@@ -4066,7 +4095,7 @@
       </c>
       <c r="AQ24" s="22">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AR24" s="27"/>
     </row>
@@ -4232,7 +4261,7 @@
       </c>
       <c r="AQ26" s="22">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR26" s="27"/>
     </row>
@@ -6213,11 +6242,11 @@
       <c r="AA64" s="129"/>
       <c r="AB64" s="130"/>
       <c r="AC64" s="39"/>
-      <c r="AD64" s="220" t="s">
+      <c r="AD64" s="218" t="s">
         <v>120</v>
       </c>
-      <c r="AE64" s="221"/>
-      <c r="AF64" s="222"/>
+      <c r="AE64" s="219"/>
+      <c r="AF64" s="220"/>
       <c r="AG64" s="39"/>
       <c r="AH64" s="78"/>
       <c r="AI64" s="79"/>
@@ -6421,9 +6450,11 @@
       <c r="AE68" s="132"/>
       <c r="AF68" s="59"/>
       <c r="AG68" s="33"/>
-      <c r="AH68" s="91"/>
-      <c r="AI68" s="92"/>
-      <c r="AJ68" s="31"/>
+      <c r="AH68" s="139" t="s">
+        <v>133</v>
+      </c>
+      <c r="AI68" s="140"/>
+      <c r="AJ68" s="68"/>
       <c r="AK68" s="29"/>
       <c r="AL68" s="139" t="s">
         <v>116</v>
@@ -6557,9 +6588,11 @@
       <c r="AE70" s="89"/>
       <c r="AF70" s="90"/>
       <c r="AG70" s="28"/>
-      <c r="AH70" s="98"/>
-      <c r="AI70" s="99"/>
-      <c r="AJ70" s="100"/>
+      <c r="AH70" s="88" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI70" s="89"/>
+      <c r="AJ70" s="90"/>
       <c r="AK70" s="29"/>
       <c r="AL70" s="208" t="s">
         <v>118</v>
@@ -6627,7 +6660,9 @@
       <c r="AE71" s="115"/>
       <c r="AF71" s="116"/>
       <c r="AG71" s="29"/>
-      <c r="AH71" s="75"/>
+      <c r="AH71" s="75" t="s">
+        <v>19</v>
+      </c>
       <c r="AI71" s="76"/>
       <c r="AJ71" s="77"/>
       <c r="AK71" s="29"/>
@@ -6685,7 +6720,9 @@
       <c r="AE72" s="106"/>
       <c r="AF72" s="107"/>
       <c r="AG72" s="33"/>
-      <c r="AH72" s="78"/>
+      <c r="AH72" s="78" t="s">
+        <v>15</v>
+      </c>
       <c r="AI72" s="79"/>
       <c r="AJ72" s="80"/>
       <c r="AK72" s="29"/>
@@ -6965,11 +7002,11 @@
       <c r="S77" s="76"/>
       <c r="T77" s="77"/>
       <c r="U77" s="28"/>
-      <c r="V77" s="216" t="s">
+      <c r="V77" s="214" t="s">
         <v>18</v>
       </c>
-      <c r="W77" s="217"/>
-      <c r="X77" s="218"/>
+      <c r="W77" s="215"/>
+      <c r="X77" s="216"/>
       <c r="Y77" s="29"/>
       <c r="Z77" s="75" t="s">
         <v>28</v>
@@ -7235,7 +7272,7 @@
         <v>52</v>
       </c>
       <c r="W82" s="82"/>
-      <c r="X82" s="219"/>
+      <c r="X82" s="217"/>
       <c r="Y82" s="29"/>
       <c r="Z82" s="98" t="s">
         <v>52</v>
@@ -7289,17 +7326,17 @@
       <c r="S83" s="76"/>
       <c r="T83" s="77"/>
       <c r="U83" s="29"/>
-      <c r="V83" s="213" t="s">
+      <c r="V83" s="211" t="s">
         <v>120</v>
       </c>
-      <c r="W83" s="214"/>
-      <c r="X83" s="215"/>
+      <c r="W83" s="212"/>
+      <c r="X83" s="213"/>
       <c r="Y83" s="29"/>
-      <c r="Z83" s="216" t="s">
+      <c r="Z83" s="214" t="s">
         <v>12</v>
       </c>
-      <c r="AA83" s="217"/>
-      <c r="AB83" s="218"/>
+      <c r="AA83" s="215"/>
+      <c r="AB83" s="216"/>
       <c r="AC83" s="29"/>
       <c r="AD83" s="75" t="s">
         <v>15</v>
@@ -7747,11 +7784,11 @@
       <c r="AE92" s="159"/>
       <c r="AF92" s="69"/>
       <c r="AG92" s="29"/>
-      <c r="AH92" s="144" t="s">
+      <c r="AH92" s="224" t="s">
         <v>58</v>
       </c>
-      <c r="AI92" s="145"/>
-      <c r="AJ92" s="62"/>
+      <c r="AI92" s="225"/>
+      <c r="AJ92" s="226"/>
       <c r="AK92" s="29"/>
       <c r="AL92" s="91"/>
       <c r="AM92" s="92"/>
@@ -7799,11 +7836,11 @@
       <c r="AE93" s="82"/>
       <c r="AF93" s="70"/>
       <c r="AG93" s="29"/>
-      <c r="AH93" s="83" t="s">
+      <c r="AH93" s="227" t="s">
         <v>67</v>
       </c>
-      <c r="AI93" s="84"/>
-      <c r="AJ93" s="64"/>
+      <c r="AI93" s="228"/>
+      <c r="AJ93" s="229"/>
       <c r="AK93" s="32"/>
       <c r="AL93" s="95"/>
       <c r="AM93" s="96"/>
@@ -7855,11 +7892,11 @@
         <v>32</v>
       </c>
       <c r="AG94" s="29"/>
-      <c r="AH94" s="110" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI94" s="111"/>
-      <c r="AJ94" s="55" t="s">
+      <c r="AH94" s="154" t="s">
+        <v>75</v>
+      </c>
+      <c r="AI94" s="155"/>
+      <c r="AJ94" s="71" t="s">
         <v>32</v>
       </c>
       <c r="AK94" s="28"/>
@@ -7913,11 +7950,11 @@
         <v>33</v>
       </c>
       <c r="AG95" s="29"/>
-      <c r="AH95" s="112" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI95" s="113"/>
-      <c r="AJ95" s="56" t="s">
+      <c r="AH95" s="156" t="s">
+        <v>76</v>
+      </c>
+      <c r="AI95" s="157"/>
+      <c r="AJ95" s="72" t="s">
         <v>33</v>
       </c>
       <c r="AK95" s="28"/>
@@ -7971,11 +8008,11 @@
         <v>34</v>
       </c>
       <c r="AG96" s="28"/>
-      <c r="AH96" s="101" t="s">
-        <v>11</v>
-      </c>
-      <c r="AI96" s="102"/>
-      <c r="AJ96" s="56" t="s">
+      <c r="AH96" s="156" t="s">
+        <v>96</v>
+      </c>
+      <c r="AI96" s="157"/>
+      <c r="AJ96" s="72" t="s">
         <v>34</v>
       </c>
       <c r="AK96" s="29"/>
@@ -8029,11 +8066,11 @@
         <v>35</v>
       </c>
       <c r="AG97" s="28"/>
-      <c r="AH97" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AI97" s="104"/>
-      <c r="AJ97" s="56" t="s">
+      <c r="AH97" s="156" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI97" s="157"/>
+      <c r="AJ97" s="72" t="s">
         <v>35</v>
       </c>
       <c r="AK97" s="29"/>
@@ -8093,11 +8130,11 @@
         <v>35</v>
       </c>
       <c r="AG98" s="33"/>
-      <c r="AH98" s="211" t="s">
-        <v>14</v>
-      </c>
-      <c r="AI98" s="212"/>
-      <c r="AJ98" s="57" t="s">
+      <c r="AH98" s="160" t="s">
+        <v>79</v>
+      </c>
+      <c r="AI98" s="161"/>
+      <c r="AJ98" s="73" t="s">
         <v>35</v>
       </c>
       <c r="AK98" s="29"/>
@@ -9654,7 +9691,7 @@
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="AF22:AF27 AB22:AB27 P22:P27 AB94:AB98 X22:X27 T22:T27 P36:P37 D58 H59 AJ22:AJ27 AF94:AF98 AN22:AN27 AJ94:AJ98 D22:D27 D70:D75 H70:H75 H22:H27 L22:L27 L59">
       <formula1>$AP$68:$AP$71</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 J132:L133 J114:L115 B126:D127 F108:H109 B114:D115 J126:L127 J120:L121 B108:D109 R22:S27 AH8:AJ10 AH63:AJ64 AL56:AN58 Z102:AB102 N56:P58 AH71:AJ72 V83:X84 AD22:AE27 R83:T84 N83:P84 N49:P51 V42:X44 AL77:AN78 V49:X51 V63:X64 N77:P78 R8:T10 AD89:AF90 V8:X10 AH42:AJ44 R63:T64 AL89:AN90 N22:O27 N101:P102 AD83:AF84 V101:X102 Z14:AB16 Z42:AB44 R14:T16 Z34:AB37 AH14:AJ16 B95:D96 AD34:AF37 V22:W27 R95:T96 B101:D102 N63:P64 R55:T58 AD8:AF10 R89:T90 J57:L58 AL14:AN16 N8:P10 V14:X16 R34:T37 V95:X96 AH83:AJ84 Z56:AB58 Z63:AB65 V56:X58 AL101:AN102 AL49:AN51 AL8:AN10 N42:P44 R77:T78 R42:T44 AL83:AN84 AD71:AF72 Z71:AB72 Z83:AB84 AH34:AJ37 AD63:AF65 AH77:AJ78 J59:K59 N14:P16 AL95:AN96 AH102:AJ102 V34:X37 N89:P90 AD94:AE98 N34:P35 AD42:AF44 Z89:AB90 Z94:AA98 AH22:AI27 V89:X90 R71:T72 Z49:AB51 V71:X72 Z22:AA27 AL22:AM27 AH49:AJ51 Z77:AB78 AL71:AN72 N71:P72 Z8:AB10 AD77:AF78 AD14:AF16 R101:T102 R49:T50 N95:P96 AL63:AN64 V77:X78 AL42:AN44 AH56:AJ58 AH94:AI98 AD49:AF51 B58:C58 N36:O37 F101:H102 B22:C27 F95:H96 B14:D16 F22:G27 B83:D84 F14:H16 F63:H64 F89:H90 B42:D44 B70:C75 B89:D90 B49:D51 F59:G59 AD102:AF102 B63:D64 F51:H52 B8:D10 F42:H46 F83:H84 B34:D37 F8:H10 F34:H37 AH89:AJ90 F70:G75 F57:H58 B56:D57 J95:L96 J101:L102 J77:L78 J8:L10 J22:K27 J63:L64 J34:L37 J83:L84 J42:L46 J14:L16 J89:L90 J71:L72 J51:L52 AL34:AN37 AD56:AF58">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 J132:L133 J114:L115 B126:D127 F108:H109 B114:D115 J126:L127 J120:L121 B108:D109 R22:S27 AH8:AJ10 AH63:AJ64 AL56:AN58 Z102:AB102 N56:P58 AD56:AF58 V83:X84 AD22:AE27 R83:T84 N83:P84 N49:P51 V42:X44 AL77:AN78 V49:X51 V63:X64 N77:P78 R8:T10 AD89:AF90 V8:X10 AH42:AJ44 R63:T64 AL89:AN90 N22:O27 N101:P102 AD83:AF84 V101:X102 Z14:AB16 Z42:AB44 R14:T16 Z34:AB37 AH14:AJ16 B95:D96 AD34:AF37 V22:W27 R95:T96 B101:D102 N63:P64 R55:T58 AD8:AF10 R89:T90 J57:L58 AL14:AN16 N8:P10 V14:X16 R34:T37 V95:X96 AH83:AJ84 Z56:AB58 Z63:AB65 V56:X58 AL101:AN102 AL49:AN51 AL8:AN10 N42:P44 R77:T78 R42:T44 AL83:AN84 AD71:AF72 Z71:AB72 Z83:AB84 AH34:AJ37 AD63:AF65 AH77:AJ78 J59:K59 N14:P16 AL95:AN96 AH102:AJ102 V34:X37 N89:P90 AD94:AE98 N34:P35 AD42:AF44 Z89:AB90 Z94:AA98 AH71:AJ72 V89:X90 R71:T72 Z49:AB51 V71:X72 Z22:AA27 AL22:AM27 AH49:AJ51 Z77:AB78 AL71:AN72 N71:P72 Z8:AB10 AD77:AF78 AD14:AF16 R101:T102 R49:T50 N95:P96 AL63:AN64 V77:X78 AL42:AN44 AH56:AJ58 AH94:AI98 AD49:AF51 B58:C58 N36:O37 F101:H102 B22:C27 F95:H96 B14:D16 F22:G27 B83:D84 F14:H16 F63:H64 F89:H90 B42:D44 B70:C75 B89:D90 B49:D51 F59:G59 AD102:AF102 B63:D64 F51:H52 B8:D10 F42:H46 F83:H84 B34:D37 F8:H10 F34:H37 AH89:AJ90 F70:G75 F57:H58 B56:D57 J95:L96 J101:L102 J77:L78 J8:L10 J22:K27 J63:L64 J34:L37 J83:L84 J42:L46 J14:L16 J89:L90 J71:L72 J51:L52 AL34:AN37 AH22:AI27">
       <formula1>$AP$6:$AP$30</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>